<commit_message>
Integrate final Janssens AISI316L workbook and reconcile overlay
</commit_message>
<xml_diff>
--- a/Experimental_Data/8_AISI316L.xlsx
+++ b/Experimental_Data/8_AISI316L.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11011"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kgfj/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{174E6DE3-DB97-4FD1-A7AA-6FFFDEFC9A5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D63E63D8-5B2F-E64B-8317-4E25AF6F45AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="189" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30260" yWindow="4360" windowWidth="38000" windowHeight="34760" tabRatio="189" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -1442,7 +1442,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normale" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="60">
     <dxf>
@@ -1782,7 +1782,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="it-IT"/>
+  <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -1864,7 +1864,7 @@
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="86"/>
                 <c:pt idx="0">
-                  <c:v>11000000</c:v>
+                  <c:v>17225000</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>2474000</c:v>
@@ -3794,24 +3794,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M28"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="27.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="68.44140625" customWidth="1"/>
+    <col min="1" max="1" width="29.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="68.5" customWidth="1"/>
     <col min="3" max="3" width="42.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="31.6640625" customWidth="1"/>
-    <col min="5" max="5" width="41.77734375" customWidth="1"/>
-    <col min="6" max="6" width="31.109375" customWidth="1"/>
+    <col min="5" max="5" width="41.83203125" customWidth="1"/>
+    <col min="6" max="6" width="31.1640625" customWidth="1"/>
     <col min="7" max="7" width="35" customWidth="1"/>
-    <col min="8" max="8" width="33.109375" customWidth="1"/>
+    <col min="8" max="8" width="33.1640625" customWidth="1"/>
     <col min="9" max="9" width="38" customWidth="1"/>
-    <col min="10" max="10" width="40.77734375" customWidth="1"/>
-    <col min="11" max="11" width="41.109375" customWidth="1"/>
+    <col min="10" max="10" width="40.83203125" customWidth="1"/>
+    <col min="11" max="11" width="41.1640625" customWidth="1"/>
     <col min="12" max="12" width="30.6640625" customWidth="1"/>
-    <col min="13" max="13" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="9.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>59</v>
       </c>
@@ -3852,7 +3852,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>95</v>
       </c>
@@ -3878,7 +3878,7 @@
         <v>265</v>
       </c>
       <c r="I2" s="1">
-        <v>241</v>
+        <v>278.5</v>
       </c>
       <c r="J2" s="1">
         <v>144</v>
@@ -3891,10 +3891,10 @@
       </c>
       <c r="M2" s="14">
         <f>IF(COUNTIF(Tabella1[[#This Row],[Tensile fatigue limit (MPa)]:[Torsional fatigue limit (MPa)]],"Null")&gt;0, "Null", IF(COUNT(Tabella1[[#This Row],[Tensile fatigue limit (MPa)]:[Torsional fatigue limit (MPa)]])=0, "Null", Tabella1[[#This Row],[Tensile fatigue limit (MPa)]]/Tabella1[[#This Row],[Torsional fatigue limit (MPa)]]))</f>
-        <v>1.6736111111111112</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+        <v>1.9340277777777777</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="13" t="s">
         <v>93</v>
       </c>
@@ -3936,7 +3936,7 @@
         <v>Null</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="13"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
@@ -3951,7 +3951,7 @@
       <c r="L4" s="1"/>
       <c r="M4" s="14"/>
     </row>
-    <row r="5" spans="1:13" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:13" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
@@ -3966,7 +3966,7 @@
       <c r="L5" s="1"/>
       <c r="M5" s="14"/>
     </row>
-    <row r="6" spans="1:13" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="59" t="s">
         <v>24</v>
       </c>
@@ -3991,7 +3991,7 @@
       </c>
       <c r="I6" s="3">
         <f>IF(COUNT(Tabella1[Tensile fatigue limit (MPa)])=0, "Null", AVERAGE(Tabella1[Tensile fatigue limit (MPa)]))</f>
-        <v>314.39999999999998</v>
+        <v>333.15</v>
       </c>
       <c r="J6" s="3">
         <f>IF(COUNT(Tabella1[Torsional fatigue limit (MPa)])=0, "Null", AVERAGE(Tabella1[Torsional fatigue limit (MPa)]))</f>
@@ -4001,10 +4001,10 @@
       <c r="L6" s="9"/>
       <c r="M6" s="15">
         <f>IF(COUNT(Tabella1[K])=0, "Null", AVERAGE(Tabella1[K]))</f>
-        <v>1.6736111111111112</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+        <v>1.9340277777777777</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="62" t="s">
         <v>23</v>
       </c>
@@ -4029,7 +4029,7 @@
       </c>
       <c r="I7" s="4">
         <f>IF(COUNT(Tabella1[Tensile fatigue limit (MPa)])=0, "Null", _xlfn.STDEV.P(Tabella1[Tensile fatigue limit (MPa)]))</f>
-        <v>73.400000000000077</v>
+        <v>54.650000000000112</v>
       </c>
       <c r="J7" s="4">
         <f>IF(COUNT(Tabella1[Torsional fatigue limit (MPa)])=0, "Null", _xlfn.STDEV.P(Tabella1[Torsional fatigue limit (MPa)]))</f>
@@ -4042,12 +4042,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="9" spans="1:13" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="10" spans="1:13" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="11" spans="1:13" ht="19.95" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="12" spans="1:13" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="13" spans="1:13" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="9" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="10" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="11" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="12" spans="1:13" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="1:13" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="65" t="s">
         <v>29</v>
       </c>
@@ -4055,18 +4055,18 @@
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:13" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A14" s="66"/>
       <c r="B14" s="6" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D27" s="7" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="28" spans="4:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D28" s="8">
         <f>COUNTA(Tabella2[Authors])</f>
         <v>86</v>
@@ -4092,55 +4092,55 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{068B26AA-516E-43B0-A4A2-503832E5DF1E}">
   <dimension ref="A1:AQ257"/>
-  <sheetFormatPr defaultColWidth="52.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="52.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="29.44140625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="29.5" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.33203125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="37.109375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="30.109375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="32.77734375" style="14" customWidth="1"/>
-    <col min="6" max="6" width="24.44140625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="49.109375" style="21" customWidth="1"/>
+    <col min="3" max="3" width="37.1640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="30.1640625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="32.83203125" style="14" customWidth="1"/>
+    <col min="6" max="6" width="24.5" style="1" customWidth="1"/>
+    <col min="7" max="7" width="49.1640625" style="21" customWidth="1"/>
     <col min="8" max="8" width="28.6640625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="63.44140625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="63.5" style="1" customWidth="1"/>
     <col min="10" max="10" width="31.33203125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="26.44140625" style="1" customWidth="1"/>
+    <col min="11" max="11" width="26.5" style="1" customWidth="1"/>
     <col min="12" max="12" width="28" style="1" customWidth="1"/>
     <col min="13" max="13" width="35" style="1" customWidth="1"/>
-    <col min="14" max="14" width="31.77734375" style="1" customWidth="1"/>
+    <col min="14" max="14" width="31.83203125" style="1" customWidth="1"/>
     <col min="15" max="15" width="35" style="1" customWidth="1"/>
-    <col min="16" max="16" width="49.44140625" style="1" customWidth="1"/>
-    <col min="17" max="17" width="53.109375" style="21" customWidth="1"/>
-    <col min="18" max="18" width="42.109375" style="1" customWidth="1"/>
-    <col min="19" max="19" width="33.44140625" style="1" customWidth="1"/>
-    <col min="20" max="20" width="38.44140625" style="1" customWidth="1"/>
-    <col min="21" max="21" width="37.109375" style="28" customWidth="1"/>
+    <col min="16" max="16" width="49.5" style="1" customWidth="1"/>
+    <col min="17" max="17" width="53.1640625" style="21" customWidth="1"/>
+    <col min="18" max="18" width="42.1640625" style="1" customWidth="1"/>
+    <col min="19" max="19" width="33.5" style="1" customWidth="1"/>
+    <col min="20" max="20" width="38.5" style="1" customWidth="1"/>
+    <col min="21" max="21" width="37.1640625" style="28" customWidth="1"/>
     <col min="22" max="22" width="40.6640625" style="28" customWidth="1"/>
     <col min="23" max="23" width="40" style="28" customWidth="1"/>
-    <col min="24" max="24" width="35.109375" style="1" customWidth="1"/>
+    <col min="24" max="24" width="35.1640625" style="1" customWidth="1"/>
     <col min="25" max="25" width="34.33203125" style="1" customWidth="1"/>
-    <col min="26" max="26" width="41.44140625" style="1" customWidth="1"/>
+    <col min="26" max="26" width="41.5" style="1" customWidth="1"/>
     <col min="27" max="27" width="28.6640625" style="49" customWidth="1"/>
-    <col min="28" max="28" width="29.44140625" style="29" customWidth="1"/>
-    <col min="29" max="29" width="27.44140625" style="29" customWidth="1"/>
-    <col min="30" max="30" width="30.109375" style="29" customWidth="1"/>
-    <col min="31" max="31" width="30.77734375" style="33" customWidth="1"/>
+    <col min="28" max="28" width="29.5" style="29" customWidth="1"/>
+    <col min="29" max="29" width="27.5" style="29" customWidth="1"/>
+    <col min="30" max="30" width="30.1640625" style="29" customWidth="1"/>
+    <col min="31" max="31" width="30.83203125" style="33" customWidth="1"/>
     <col min="32" max="32" width="25" style="29" customWidth="1"/>
     <col min="33" max="33" width="30.33203125" style="21" customWidth="1"/>
-    <col min="34" max="34" width="28.44140625" style="29" customWidth="1"/>
+    <col min="34" max="34" width="28.5" style="29" customWidth="1"/>
     <col min="35" max="35" width="29.33203125" style="29" customWidth="1"/>
-    <col min="36" max="36" width="20.109375" style="29" customWidth="1"/>
-    <col min="37" max="37" width="23.109375" style="29" customWidth="1"/>
+    <col min="36" max="36" width="20.1640625" style="29" customWidth="1"/>
+    <col min="37" max="37" width="23.1640625" style="29" customWidth="1"/>
     <col min="38" max="38" width="23.33203125" style="29" customWidth="1"/>
-    <col min="39" max="39" width="25.77734375" style="29" customWidth="1"/>
-    <col min="40" max="40" width="23.77734375" style="29" customWidth="1"/>
+    <col min="39" max="39" width="25.83203125" style="29" customWidth="1"/>
+    <col min="40" max="40" width="23.83203125" style="29" customWidth="1"/>
     <col min="41" max="41" width="24" style="23" customWidth="1"/>
-    <col min="42" max="42" width="25.77734375" style="21" customWidth="1"/>
+    <col min="42" max="42" width="25.83203125" style="21" customWidth="1"/>
     <col min="43" max="43" width="27.6640625" style="41" customWidth="1"/>
     <col min="44" max="16384" width="52.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" s="27" customFormat="1" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:43" s="27" customFormat="1" ht="44.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="26" t="s">
         <v>26</v>
       </c>
@@ -4271,7 +4271,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>62</v>
       </c>
@@ -4285,7 +4285,7 @@
         <v>64</v>
       </c>
       <c r="E2" s="28">
-        <v>11000000</v>
+        <v>17225000</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>32</v>
@@ -4448,7 +4448,7 @@
         <v>265.8</v>
       </c>
     </row>
-    <row r="3" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>62</v>
       </c>
@@ -4625,7 +4625,7 @@
         <v>271.60000000000002</v>
       </c>
     </row>
-    <row r="4" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>62</v>
       </c>
@@ -4802,7 +4802,7 @@
         <v>271.60000000000002</v>
       </c>
     </row>
-    <row r="5" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>62</v>
       </c>
@@ -4979,7 +4979,7 @@
         <v>271.60000000000002</v>
       </c>
     </row>
-    <row r="6" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>62</v>
       </c>
@@ -5156,7 +5156,7 @@
         <v>277.39999999999998</v>
       </c>
     </row>
-    <row r="7" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>62</v>
       </c>
@@ -5333,7 +5333,7 @@
         <v>277.39999999999998</v>
       </c>
     </row>
-    <row r="8" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>62</v>
       </c>
@@ -5510,7 +5510,7 @@
         <v>277.39999999999998</v>
       </c>
     </row>
-    <row r="9" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>62</v>
       </c>
@@ -5687,7 +5687,7 @@
         <v>283.2</v>
       </c>
     </row>
-    <row r="10" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>62</v>
       </c>
@@ -5864,7 +5864,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="11" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>62</v>
       </c>
@@ -6041,7 +6041,7 @@
         <v>240.06224192904639</v>
       </c>
     </row>
-    <row r="12" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>62</v>
       </c>
@@ -6218,7 +6218,7 @@
         <v>249.93493153218898</v>
       </c>
     </row>
-    <row r="13" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>62</v>
       </c>
@@ -6395,7 +6395,7 @@
         <v>249.93493153218898</v>
       </c>
     </row>
-    <row r="14" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>62</v>
       </c>
@@ -6572,7 +6572,7 @@
         <v>249.93493153218898</v>
       </c>
     </row>
-    <row r="15" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>62</v>
       </c>
@@ -6749,7 +6749,7 @@
         <v>254.95787887413871</v>
       </c>
     </row>
-    <row r="16" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>62</v>
       </c>
@@ -6926,7 +6926,7 @@
         <v>259.98082621608847</v>
       </c>
     </row>
-    <row r="17" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>62</v>
       </c>
@@ -7103,7 +7103,7 @@
         <v>265.00377355803823</v>
       </c>
     </row>
-    <row r="18" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>62</v>
       </c>
@@ -7192,7 +7192,7 @@
         <v>0</v>
       </c>
       <c r="T18" s="1">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="U18" s="28">
         <v>10</v>
@@ -7280,7 +7280,7 @@
         <v>259.35922964105208</v>
       </c>
     </row>
-    <row r="19" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>62</v>
       </c>
@@ -7369,7 +7369,7 @@
         <v>0</v>
       </c>
       <c r="T19" s="1">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="U19" s="28">
         <v>10</v>
@@ -7457,7 +7457,7 @@
         <v>280.94106143460056</v>
       </c>
     </row>
-    <row r="20" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>62</v>
       </c>
@@ -7546,7 +7546,7 @@
         <v>0</v>
       </c>
       <c r="T20" s="1">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="U20" s="28">
         <v>10</v>
@@ -7634,7 +7634,7 @@
         <v>291.71300965160947</v>
       </c>
     </row>
-    <row r="21" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>62</v>
       </c>
@@ -7723,7 +7723,7 @@
         <v>0</v>
       </c>
       <c r="T21" s="1">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="U21" s="28">
         <v>10</v>
@@ -7811,7 +7811,7 @@
         <v>302.56058897351454</v>
       </c>
     </row>
-    <row r="22" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>62</v>
       </c>
@@ -7900,7 +7900,7 @@
         <v>0</v>
       </c>
       <c r="T22" s="1">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="U22" s="28">
         <v>10</v>
@@ -7988,7 +7988,7 @@
         <v>313.33255496357225</v>
       </c>
     </row>
-    <row r="23" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>62</v>
       </c>
@@ -8077,7 +8077,7 @@
         <v>0</v>
       </c>
       <c r="T23" s="1">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="U23" s="28">
         <v>10</v>
@@ -8165,7 +8165,7 @@
         <v>320.89189768518617</v>
       </c>
     </row>
-    <row r="24" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
         <v>62</v>
       </c>
@@ -8254,7 +8254,7 @@
         <v>0</v>
       </c>
       <c r="T24" s="1">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="U24" s="28">
         <v>10</v>
@@ -8342,7 +8342,7 @@
         <v>324.18013511009582</v>
       </c>
     </row>
-    <row r="25" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
         <v>62</v>
       </c>
@@ -8431,7 +8431,7 @@
         <v>0</v>
       </c>
       <c r="T25" s="1">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="U25" s="28">
         <v>10</v>
@@ -8519,7 +8519,7 @@
         <v>328.56457508380294</v>
       </c>
     </row>
-    <row r="26" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
         <v>62</v>
       </c>
@@ -8608,7 +8608,7 @@
         <v>0</v>
       </c>
       <c r="T26" s="1">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="U26" s="28">
         <v>10</v>
@@ -8696,7 +8696,7 @@
         <v>335.10332734844633</v>
       </c>
     </row>
-    <row r="27" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
         <v>62</v>
       </c>
@@ -8785,7 +8785,7 @@
         <v>0</v>
       </c>
       <c r="T27" s="1">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="U27" s="28">
         <v>10</v>
@@ -8873,7 +8873,7 @@
         <v>336.23725254647201</v>
       </c>
     </row>
-    <row r="28" spans="1:43" s="17" customFormat="1" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:43" s="17" customFormat="1" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A28" s="17" t="s">
         <v>62</v>
       </c>
@@ -8962,7 +8962,7 @@
         <v>0</v>
       </c>
       <c r="T28" s="17">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="U28" s="18">
         <v>1</v>
@@ -9050,7 +9050,7 @@
         <v>345.950906921777</v>
       </c>
     </row>
-    <row r="29" spans="1:43" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:43" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
         <v>94</v>
       </c>
@@ -9227,7 +9227,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="30" spans="1:43" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:43" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
         <v>94</v>
       </c>
@@ -9404,7 +9404,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="31" spans="1:43" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:43" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
         <v>94</v>
       </c>
@@ -9581,7 +9581,7 @@
         <v>108.5</v>
       </c>
     </row>
-    <row r="32" spans="1:43" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:43" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
         <v>94</v>
       </c>
@@ -9758,7 +9758,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="33" spans="1:43" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:43" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
         <v>94</v>
       </c>
@@ -9935,7 +9935,7 @@
         <v>108.5</v>
       </c>
     </row>
-    <row r="34" spans="1:43" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:43" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
         <v>94</v>
       </c>
@@ -10112,7 +10112,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="35" spans="1:43" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:43" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
         <v>94</v>
       </c>
@@ -10289,7 +10289,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="36" spans="1:43" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:43" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
         <v>94</v>
       </c>
@@ -10466,7 +10466,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="37" spans="1:43" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:43" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
         <v>94</v>
       </c>
@@ -10643,7 +10643,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="38" spans="1:43" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:43" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
         <v>94</v>
       </c>
@@ -10820,7 +10820,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="39" spans="1:43" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:43" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
         <v>94</v>
       </c>
@@ -10997,7 +10997,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="40" spans="1:43" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:43" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
         <v>94</v>
       </c>
@@ -11174,7 +11174,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="41" spans="1:43" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:43" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
         <v>94</v>
       </c>
@@ -11351,7 +11351,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="42" spans="1:43" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:43" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
         <v>94</v>
       </c>
@@ -11528,7 +11528,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="43" spans="1:43" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:43" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
         <v>94</v>
       </c>
@@ -11705,7 +11705,7 @@
         <v>91.5</v>
       </c>
     </row>
-    <row r="44" spans="1:43" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:43" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
         <v>94</v>
       </c>
@@ -11882,7 +11882,7 @@
         <v>91.5</v>
       </c>
     </row>
-    <row r="45" spans="1:43" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:43" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
         <v>94</v>
       </c>
@@ -12059,7 +12059,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="46" spans="1:43" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:43" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
         <v>94</v>
       </c>
@@ -12236,7 +12236,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="47" spans="1:43" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:43" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
         <v>94</v>
       </c>
@@ -12413,7 +12413,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="48" spans="1:43" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:43" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
         <v>94</v>
       </c>
@@ -12590,7 +12590,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="49" spans="1:43" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:43" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
         <v>94</v>
       </c>
@@ -12767,7 +12767,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="50" spans="1:43" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:43" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
         <v>94</v>
       </c>
@@ -12944,7 +12944,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="51" spans="1:43" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:43" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
         <v>94</v>
       </c>
@@ -13121,7 +13121,7 @@
         <v>158.5</v>
       </c>
     </row>
-    <row r="52" spans="1:43" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:43" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
         <v>94</v>
       </c>
@@ -13298,7 +13298,7 @@
         <v>158.5</v>
       </c>
     </row>
-    <row r="53" spans="1:43" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:43" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
         <v>94</v>
       </c>
@@ -13475,7 +13475,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="54" spans="1:43" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:43" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
         <v>94</v>
       </c>
@@ -13652,7 +13652,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="55" spans="1:43" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:43" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
         <v>94</v>
       </c>
@@ -13829,7 +13829,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="56" spans="1:43" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:43" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
         <v>94</v>
       </c>
@@ -14006,7 +14006,7 @@
         <v>146.5</v>
       </c>
     </row>
-    <row r="57" spans="1:43" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:43" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
         <v>94</v>
       </c>
@@ -14183,7 +14183,7 @@
         <v>137.5</v>
       </c>
     </row>
-    <row r="58" spans="1:43" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:43" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
         <v>94</v>
       </c>
@@ -14360,7 +14360,7 @@
         <v>133.5</v>
       </c>
     </row>
-    <row r="59" spans="1:43" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:43" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
         <v>94</v>
       </c>
@@ -14537,7 +14537,7 @@
         <v>141.5</v>
       </c>
     </row>
-    <row r="60" spans="1:43" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:43" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
         <v>94</v>
       </c>
@@ -14714,7 +14714,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="61" spans="1:43" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:43" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
         <v>94</v>
       </c>
@@ -14891,7 +14891,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="62" spans="1:43" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:43" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="1" t="s">
         <v>94</v>
       </c>
@@ -15068,7 +15068,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="63" spans="1:43" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:43" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="s">
         <v>94</v>
       </c>
@@ -15245,7 +15245,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="64" spans="1:43" customFormat="1" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:43" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
         <v>94</v>
       </c>
@@ -15422,7 +15422,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="65" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
         <v>94</v>
       </c>
@@ -15599,7 +15599,7 @@
         <v>137.5</v>
       </c>
     </row>
-    <row r="66" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="1" t="s">
         <v>94</v>
       </c>
@@ -15776,7 +15776,7 @@
         <v>133.5</v>
       </c>
     </row>
-    <row r="67" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="1" t="s">
         <v>94</v>
       </c>
@@ -15953,7 +15953,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="68" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="1" t="s">
         <v>94</v>
       </c>
@@ -16130,7 +16130,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="69" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="1" t="s">
         <v>94</v>
       </c>
@@ -16307,7 +16307,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="70" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="1" t="s">
         <v>94</v>
       </c>
@@ -16484,7 +16484,7 @@
         <v>137.5</v>
       </c>
     </row>
-    <row r="71" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="1" t="s">
         <v>94</v>
       </c>
@@ -16661,7 +16661,7 @@
         <v>255.717949373556</v>
       </c>
     </row>
-    <row r="72" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="1" t="s">
         <v>94</v>
       </c>
@@ -16838,7 +16838,7 @@
         <v>240.04280092058249</v>
       </c>
     </row>
-    <row r="73" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="1" t="s">
         <v>94</v>
       </c>
@@ -17015,7 +17015,7 @@
         <v>248.279407501717</v>
       </c>
     </row>
-    <row r="74" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="1" t="s">
         <v>94</v>
       </c>
@@ -17192,7 +17192,7 @@
         <v>241.05724428188401</v>
       </c>
     </row>
-    <row r="75" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="1" t="s">
         <v>94</v>
       </c>
@@ -17369,7 +17369,7 @@
         <v>249.32865953394651</v>
       </c>
     </row>
-    <row r="76" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="1" t="s">
         <v>94</v>
       </c>
@@ -17546,7 +17546,7 @@
         <v>251.4404850500205</v>
       </c>
     </row>
-    <row r="77" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="1" t="s">
         <v>94</v>
       </c>
@@ -17723,7 +17723,7 @@
         <v>241.05724428188401</v>
       </c>
     </row>
-    <row r="78" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="1" t="s">
         <v>94</v>
       </c>
@@ -17900,7 +17900,7 @@
         <v>224.38026487041699</v>
       </c>
     </row>
-    <row r="79" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="1" t="s">
         <v>94</v>
       </c>
@@ -18077,7 +18077,7 @@
         <v>224.38026487041699</v>
       </c>
     </row>
-    <row r="80" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="1" t="s">
         <v>94</v>
       </c>
@@ -18254,7 +18254,7 @@
         <v>209.739692547478</v>
       </c>
     </row>
-    <row r="81" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="1" t="s">
         <v>94</v>
       </c>
@@ -18431,7 +18431,7 @@
         <v>226.28077630597551</v>
       </c>
     </row>
-    <row r="82" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="1" t="s">
         <v>94</v>
       </c>
@@ -18608,7 +18608,7 @@
         <v>225.32851688727351</v>
       </c>
     </row>
-    <row r="83" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="1" t="s">
         <v>94</v>
       </c>
@@ -18785,7 +18785,7 @@
         <v>224.38026487041699</v>
       </c>
     </row>
-    <row r="84" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="1" t="s">
         <v>94</v>
       </c>
@@ -18962,7 +18962,7 @@
         <v>242.07597477585199</v>
       </c>
     </row>
-    <row r="85" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="1" t="s">
         <v>94</v>
       </c>
@@ -19139,7 +19139,7 @@
         <v>215.11447653364851</v>
       </c>
     </row>
-    <row r="86" spans="1:43" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:43" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="1" t="s">
         <v>94</v>
       </c>
@@ -19316,7 +19316,7 @@
         <v>205.363434036618</v>
       </c>
     </row>
-    <row r="87" spans="1:43" s="17" customFormat="1" ht="19.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:43" s="17" customFormat="1" ht="20" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A87" s="17" t="s">
         <v>94</v>
       </c>
@@ -19493,13 +19493,13 @@
         <v>198.550554026415</v>
       </c>
     </row>
-    <row r="88" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:43" x14ac:dyDescent="0.2">
       <c r="O88" s="28"/>
       <c r="P88" s="28"/>
       <c r="Z88" s="29"/>
       <c r="AG88" s="24"/>
     </row>
-    <row r="89" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:43" x14ac:dyDescent="0.2">
       <c r="G89" s="1"/>
       <c r="O89" s="28"/>
       <c r="P89" s="28"/>
@@ -19511,7 +19511,7 @@
       <c r="AP89" s="1"/>
       <c r="AQ89" s="14"/>
     </row>
-    <row r="90" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:43" x14ac:dyDescent="0.2">
       <c r="G90" s="1"/>
       <c r="O90" s="28"/>
       <c r="P90" s="28"/>
@@ -19523,7 +19523,7 @@
       <c r="AP90" s="1"/>
       <c r="AQ90" s="14"/>
     </row>
-    <row r="91" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:43" x14ac:dyDescent="0.2">
       <c r="G91" s="1"/>
       <c r="O91" s="28"/>
       <c r="P91" s="28"/>
@@ -19535,7 +19535,7 @@
       <c r="AP91" s="1"/>
       <c r="AQ91" s="14"/>
     </row>
-    <row r="92" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:43" x14ac:dyDescent="0.2">
       <c r="G92" s="1"/>
       <c r="O92" s="28"/>
       <c r="P92" s="28"/>
@@ -19547,7 +19547,7 @@
       <c r="AP92" s="1"/>
       <c r="AQ92" s="14"/>
     </row>
-    <row r="93" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:43" x14ac:dyDescent="0.2">
       <c r="G93" s="1"/>
       <c r="O93" s="28"/>
       <c r="P93" s="28"/>
@@ -19559,7 +19559,7 @@
       <c r="AP93" s="1"/>
       <c r="AQ93" s="14"/>
     </row>
-    <row r="94" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:43" x14ac:dyDescent="0.2">
       <c r="G94" s="1"/>
       <c r="O94" s="28"/>
       <c r="P94" s="28"/>
@@ -19571,7 +19571,7 @@
       <c r="AP94" s="1"/>
       <c r="AQ94" s="14"/>
     </row>
-    <row r="95" spans="1:43" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:43" x14ac:dyDescent="0.2">
       <c r="G95" s="1"/>
       <c r="O95" s="28"/>
       <c r="P95" s="28"/>
@@ -19583,7 +19583,7 @@
       <c r="AP95" s="1"/>
       <c r="AQ95" s="14"/>
     </row>
-    <row r="96" spans="1:43" ht="17.55" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:43" ht="17.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="G96" s="1"/>
       <c r="O96" s="28"/>
       <c r="P96" s="28"/>
@@ -19595,7 +19595,7 @@
       <c r="AP96" s="1"/>
       <c r="AQ96" s="14"/>
     </row>
-    <row r="97" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="97" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G97" s="1"/>
       <c r="O97" s="28"/>
       <c r="P97" s="28"/>
@@ -19607,7 +19607,7 @@
       <c r="AP97" s="1"/>
       <c r="AQ97" s="14"/>
     </row>
-    <row r="98" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="98" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G98" s="1"/>
       <c r="O98" s="28"/>
       <c r="P98" s="28"/>
@@ -19619,7 +19619,7 @@
       <c r="AP98" s="1"/>
       <c r="AQ98" s="14"/>
     </row>
-    <row r="99" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="99" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G99" s="1"/>
       <c r="O99" s="28"/>
       <c r="P99" s="28"/>
@@ -19631,7 +19631,7 @@
       <c r="AP99" s="1"/>
       <c r="AQ99" s="14"/>
     </row>
-    <row r="100" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="100" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G100" s="1"/>
       <c r="O100" s="28"/>
       <c r="P100" s="28"/>
@@ -19645,7 +19645,7 @@
       <c r="AP100" s="1"/>
       <c r="AQ100" s="14"/>
     </row>
-    <row r="101" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="101" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G101" s="1"/>
       <c r="O101" s="28"/>
       <c r="P101" s="28"/>
@@ -19659,7 +19659,7 @@
       <c r="AP101" s="1"/>
       <c r="AQ101" s="14"/>
     </row>
-    <row r="102" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="102" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G102" s="1"/>
       <c r="O102" s="28"/>
       <c r="P102" s="28"/>
@@ -19673,7 +19673,7 @@
       <c r="AP102" s="1"/>
       <c r="AQ102" s="14"/>
     </row>
-    <row r="103" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="103" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G103" s="1"/>
       <c r="O103" s="28"/>
       <c r="P103" s="28"/>
@@ -19687,7 +19687,7 @@
       <c r="AP103" s="1"/>
       <c r="AQ103" s="14"/>
     </row>
-    <row r="104" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="104" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G104" s="1"/>
       <c r="O104" s="28"/>
       <c r="P104" s="28"/>
@@ -19699,7 +19699,7 @@
       <c r="AP104" s="1"/>
       <c r="AQ104" s="14"/>
     </row>
-    <row r="105" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="105" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G105" s="1"/>
       <c r="O105" s="28"/>
       <c r="P105" s="28"/>
@@ -19711,7 +19711,7 @@
       <c r="AP105" s="1"/>
       <c r="AQ105" s="14"/>
     </row>
-    <row r="106" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="106" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G106" s="1"/>
       <c r="O106" s="28"/>
       <c r="P106" s="28"/>
@@ -19723,7 +19723,7 @@
       <c r="AP106" s="1"/>
       <c r="AQ106" s="14"/>
     </row>
-    <row r="107" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="107" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G107" s="1"/>
       <c r="O107" s="28"/>
       <c r="P107" s="28"/>
@@ -19735,7 +19735,7 @@
       <c r="AP107" s="1"/>
       <c r="AQ107" s="14"/>
     </row>
-    <row r="108" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="108" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G108" s="1"/>
       <c r="O108" s="28"/>
       <c r="P108" s="28"/>
@@ -19747,7 +19747,7 @@
       <c r="AP108" s="1"/>
       <c r="AQ108" s="14"/>
     </row>
-    <row r="109" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="109" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G109" s="1"/>
       <c r="O109" s="28"/>
       <c r="P109" s="28"/>
@@ -19759,7 +19759,7 @@
       <c r="AP109" s="1"/>
       <c r="AQ109" s="14"/>
     </row>
-    <row r="110" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="110" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G110" s="1"/>
       <c r="O110" s="28"/>
       <c r="P110" s="28"/>
@@ -19771,7 +19771,7 @@
       <c r="AP110" s="1"/>
       <c r="AQ110" s="14"/>
     </row>
-    <row r="111" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="111" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G111" s="1"/>
       <c r="O111" s="28"/>
       <c r="P111" s="28"/>
@@ -19783,7 +19783,7 @@
       <c r="AP111" s="1"/>
       <c r="AQ111" s="14"/>
     </row>
-    <row r="112" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="112" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G112" s="1"/>
       <c r="O112" s="28"/>
       <c r="P112" s="28"/>
@@ -19794,7 +19794,7 @@
       <c r="AP112" s="1"/>
       <c r="AQ112" s="14"/>
     </row>
-    <row r="113" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="113" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G113" s="1"/>
       <c r="O113" s="28"/>
       <c r="P113" s="28"/>
@@ -19805,7 +19805,7 @@
       <c r="AP113" s="1"/>
       <c r="AQ113" s="14"/>
     </row>
-    <row r="114" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="114" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G114" s="1"/>
       <c r="O114" s="28"/>
       <c r="P114" s="28"/>
@@ -19816,7 +19816,7 @@
       <c r="AP114" s="1"/>
       <c r="AQ114" s="14"/>
     </row>
-    <row r="115" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="115" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G115" s="1"/>
       <c r="O115" s="28"/>
       <c r="P115" s="28"/>
@@ -19827,7 +19827,7 @@
       <c r="AP115" s="1"/>
       <c r="AQ115" s="14"/>
     </row>
-    <row r="116" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="116" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G116" s="1"/>
       <c r="O116" s="28"/>
       <c r="P116" s="28"/>
@@ -19838,7 +19838,7 @@
       <c r="AP116" s="1"/>
       <c r="AQ116" s="14"/>
     </row>
-    <row r="117" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="117" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G117" s="1"/>
       <c r="O117" s="28"/>
       <c r="P117" s="28"/>
@@ -19849,7 +19849,7 @@
       <c r="AP117" s="1"/>
       <c r="AQ117" s="14"/>
     </row>
-    <row r="118" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="118" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G118" s="1"/>
       <c r="O118" s="28"/>
       <c r="P118" s="28"/>
@@ -19860,7 +19860,7 @@
       <c r="AP118" s="1"/>
       <c r="AQ118" s="14"/>
     </row>
-    <row r="119" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="119" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G119" s="1"/>
       <c r="O119" s="28"/>
       <c r="P119" s="28"/>
@@ -19871,7 +19871,7 @@
       <c r="AP119" s="1"/>
       <c r="AQ119" s="14"/>
     </row>
-    <row r="120" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="120" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G120" s="1"/>
       <c r="O120" s="28"/>
       <c r="P120" s="28"/>
@@ -19882,7 +19882,7 @@
       <c r="AP120" s="1"/>
       <c r="AQ120" s="14"/>
     </row>
-    <row r="121" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="121" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G121" s="1"/>
       <c r="O121" s="28"/>
       <c r="P121" s="28"/>
@@ -19893,7 +19893,7 @@
       <c r="AP121" s="1"/>
       <c r="AQ121" s="14"/>
     </row>
-    <row r="122" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="122" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G122" s="1"/>
       <c r="O122" s="28"/>
       <c r="P122" s="28"/>
@@ -19904,7 +19904,7 @@
       <c r="AP122" s="1"/>
       <c r="AQ122" s="14"/>
     </row>
-    <row r="123" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="123" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G123" s="1"/>
       <c r="O123" s="28"/>
       <c r="P123" s="28"/>
@@ -19915,7 +19915,7 @@
       <c r="AP123" s="1"/>
       <c r="AQ123" s="14"/>
     </row>
-    <row r="124" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="124" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G124" s="1"/>
       <c r="O124" s="28"/>
       <c r="P124" s="28"/>
@@ -19926,7 +19926,7 @@
       <c r="AP124" s="1"/>
       <c r="AQ124" s="14"/>
     </row>
-    <row r="125" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="125" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G125" s="1"/>
       <c r="O125" s="28"/>
       <c r="P125" s="28"/>
@@ -19937,7 +19937,7 @@
       <c r="AP125" s="1"/>
       <c r="AQ125" s="14"/>
     </row>
-    <row r="126" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="126" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G126" s="1"/>
       <c r="O126" s="28"/>
       <c r="P126" s="28"/>
@@ -19948,7 +19948,7 @@
       <c r="AP126" s="1"/>
       <c r="AQ126" s="14"/>
     </row>
-    <row r="127" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="127" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G127" s="1"/>
       <c r="O127" s="28"/>
       <c r="P127" s="28"/>
@@ -19959,7 +19959,7 @@
       <c r="AP127" s="1"/>
       <c r="AQ127" s="14"/>
     </row>
-    <row r="128" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="128" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G128" s="1"/>
       <c r="O128" s="28"/>
       <c r="P128" s="28"/>
@@ -19970,7 +19970,7 @@
       <c r="AP128" s="1"/>
       <c r="AQ128" s="14"/>
     </row>
-    <row r="129" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="129" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G129" s="1"/>
       <c r="O129" s="28"/>
       <c r="P129" s="28"/>
@@ -19981,7 +19981,7 @@
       <c r="AP129" s="1"/>
       <c r="AQ129" s="14"/>
     </row>
-    <row r="130" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="130" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G130" s="1"/>
       <c r="O130" s="28"/>
       <c r="P130" s="28"/>
@@ -19992,7 +19992,7 @@
       <c r="AP130" s="1"/>
       <c r="AQ130" s="14"/>
     </row>
-    <row r="131" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="131" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G131" s="1"/>
       <c r="O131" s="28"/>
       <c r="P131" s="28"/>
@@ -20003,7 +20003,7 @@
       <c r="AP131" s="1"/>
       <c r="AQ131" s="14"/>
     </row>
-    <row r="132" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="132" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G132" s="1"/>
       <c r="O132" s="28"/>
       <c r="P132" s="28"/>
@@ -20014,7 +20014,7 @@
       <c r="AP132" s="1"/>
       <c r="AQ132" s="14"/>
     </row>
-    <row r="133" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="133" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G133" s="1"/>
       <c r="O133" s="28"/>
       <c r="P133" s="28"/>
@@ -20025,7 +20025,7 @@
       <c r="AP133" s="1"/>
       <c r="AQ133" s="14"/>
     </row>
-    <row r="134" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="134" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G134" s="1"/>
       <c r="O134" s="28"/>
       <c r="P134" s="28"/>
@@ -20036,7 +20036,7 @@
       <c r="AP134" s="1"/>
       <c r="AQ134" s="14"/>
     </row>
-    <row r="135" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="135" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G135" s="1"/>
       <c r="O135" s="28"/>
       <c r="P135" s="28"/>
@@ -20047,7 +20047,7 @@
       <c r="AP135" s="1"/>
       <c r="AQ135" s="14"/>
     </row>
-    <row r="136" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="136" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G136" s="1"/>
       <c r="O136" s="28"/>
       <c r="P136" s="28"/>
@@ -20058,7 +20058,7 @@
       <c r="AP136" s="1"/>
       <c r="AQ136" s="14"/>
     </row>
-    <row r="137" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="137" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G137" s="1"/>
       <c r="O137" s="28"/>
       <c r="P137" s="28"/>
@@ -20069,7 +20069,7 @@
       <c r="AP137" s="1"/>
       <c r="AQ137" s="14"/>
     </row>
-    <row r="138" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="138" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G138" s="1"/>
       <c r="O138" s="28"/>
       <c r="P138" s="28"/>
@@ -20080,7 +20080,7 @@
       <c r="AP138" s="1"/>
       <c r="AQ138" s="14"/>
     </row>
-    <row r="139" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="139" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G139" s="1"/>
       <c r="O139" s="28"/>
       <c r="P139" s="28"/>
@@ -20091,7 +20091,7 @@
       <c r="AP139" s="1"/>
       <c r="AQ139" s="14"/>
     </row>
-    <row r="140" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="140" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G140" s="1"/>
       <c r="O140" s="28"/>
       <c r="P140" s="28"/>
@@ -20102,7 +20102,7 @@
       <c r="AP140" s="1"/>
       <c r="AQ140" s="14"/>
     </row>
-    <row r="141" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="141" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G141" s="1"/>
       <c r="O141" s="28"/>
       <c r="P141" s="28"/>
@@ -20113,7 +20113,7 @@
       <c r="AP141" s="1"/>
       <c r="AQ141" s="14"/>
     </row>
-    <row r="142" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="142" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G142" s="1"/>
       <c r="O142" s="28"/>
       <c r="P142" s="28"/>
@@ -20124,7 +20124,7 @@
       <c r="AP142" s="1"/>
       <c r="AQ142" s="14"/>
     </row>
-    <row r="143" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="143" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G143" s="1"/>
       <c r="O143" s="28"/>
       <c r="P143" s="28"/>
@@ -20135,7 +20135,7 @@
       <c r="AP143" s="1"/>
       <c r="AQ143" s="14"/>
     </row>
-    <row r="144" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="144" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G144" s="1"/>
       <c r="O144" s="28"/>
       <c r="P144" s="28"/>
@@ -20146,7 +20146,7 @@
       <c r="AP144" s="1"/>
       <c r="AQ144" s="14"/>
     </row>
-    <row r="145" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="145" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G145" s="1"/>
       <c r="O145" s="28"/>
       <c r="P145" s="28"/>
@@ -20157,7 +20157,7 @@
       <c r="AP145" s="1"/>
       <c r="AQ145" s="14"/>
     </row>
-    <row r="146" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="146" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G146" s="1"/>
       <c r="O146" s="28"/>
       <c r="P146" s="28"/>
@@ -20168,7 +20168,7 @@
       <c r="AP146" s="1"/>
       <c r="AQ146" s="14"/>
     </row>
-    <row r="147" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="147" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G147" s="1"/>
       <c r="O147" s="28"/>
       <c r="P147" s="28"/>
@@ -20179,7 +20179,7 @@
       <c r="AP147" s="1"/>
       <c r="AQ147" s="14"/>
     </row>
-    <row r="148" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="148" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G148" s="1"/>
       <c r="O148" s="28"/>
       <c r="P148" s="28"/>
@@ -20190,7 +20190,7 @@
       <c r="AP148" s="1"/>
       <c r="AQ148" s="14"/>
     </row>
-    <row r="149" spans="7:43" ht="13.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="149" spans="7:43" ht="13.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="G149" s="1"/>
       <c r="O149" s="28"/>
       <c r="P149" s="28"/>
@@ -20201,7 +20201,7 @@
       <c r="AP149" s="1"/>
       <c r="AQ149" s="14"/>
     </row>
-    <row r="150" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="150" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G150" s="1"/>
       <c r="O150" s="28"/>
       <c r="P150" s="28"/>
@@ -20212,7 +20212,7 @@
       <c r="AP150" s="1"/>
       <c r="AQ150" s="14"/>
     </row>
-    <row r="151" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="151" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G151" s="1"/>
       <c r="O151" s="28"/>
       <c r="P151" s="28"/>
@@ -20223,7 +20223,7 @@
       <c r="AP151" s="1"/>
       <c r="AQ151" s="14"/>
     </row>
-    <row r="152" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="152" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G152" s="1"/>
       <c r="O152" s="28"/>
       <c r="P152" s="28"/>
@@ -20234,7 +20234,7 @@
       <c r="AP152" s="1"/>
       <c r="AQ152" s="14"/>
     </row>
-    <row r="153" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="153" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G153" s="1"/>
       <c r="O153" s="28"/>
       <c r="P153" s="28"/>
@@ -20245,7 +20245,7 @@
       <c r="AP153" s="1"/>
       <c r="AQ153" s="14"/>
     </row>
-    <row r="154" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="154" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G154" s="1"/>
       <c r="O154" s="28"/>
       <c r="P154" s="28"/>
@@ -20256,7 +20256,7 @@
       <c r="AP154" s="1"/>
       <c r="AQ154" s="14"/>
     </row>
-    <row r="155" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="155" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G155" s="1"/>
       <c r="O155" s="28"/>
       <c r="P155" s="28"/>
@@ -20267,7 +20267,7 @@
       <c r="AP155" s="1"/>
       <c r="AQ155" s="14"/>
     </row>
-    <row r="156" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="156" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G156" s="1"/>
       <c r="O156" s="28"/>
       <c r="P156" s="28"/>
@@ -20278,7 +20278,7 @@
       <c r="AP156" s="1"/>
       <c r="AQ156" s="14"/>
     </row>
-    <row r="157" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="157" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G157" s="1"/>
       <c r="O157" s="28"/>
       <c r="P157" s="28"/>
@@ -20289,7 +20289,7 @@
       <c r="AP157" s="1"/>
       <c r="AQ157" s="14"/>
     </row>
-    <row r="158" spans="7:43" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="158" spans="7:43" ht="14" customHeight="1" x14ac:dyDescent="0.2">
       <c r="G158" s="1"/>
       <c r="O158" s="28"/>
       <c r="P158" s="28"/>
@@ -20300,7 +20300,7 @@
       <c r="AP158" s="1"/>
       <c r="AQ158" s="14"/>
     </row>
-    <row r="159" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="159" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G159" s="1"/>
       <c r="O159" s="28"/>
       <c r="P159" s="28"/>
@@ -20311,7 +20311,7 @@
       <c r="AP159" s="1"/>
       <c r="AQ159" s="14"/>
     </row>
-    <row r="160" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="160" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G160" s="1"/>
       <c r="O160" s="28"/>
       <c r="P160" s="28"/>
@@ -20322,7 +20322,7 @@
       <c r="AP160" s="1"/>
       <c r="AQ160" s="14"/>
     </row>
-    <row r="161" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="161" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G161" s="1"/>
       <c r="O161" s="28"/>
       <c r="P161" s="28"/>
@@ -20333,7 +20333,7 @@
       <c r="AP161" s="1"/>
       <c r="AQ161" s="14"/>
     </row>
-    <row r="162" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="162" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G162" s="1"/>
       <c r="O162" s="28"/>
       <c r="P162" s="28"/>
@@ -20344,7 +20344,7 @@
       <c r="AP162" s="1"/>
       <c r="AQ162" s="14"/>
     </row>
-    <row r="163" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="163" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G163" s="1"/>
       <c r="O163" s="28"/>
       <c r="P163" s="28"/>
@@ -20355,7 +20355,7 @@
       <c r="AP163" s="1"/>
       <c r="AQ163" s="14"/>
     </row>
-    <row r="164" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="164" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G164" s="1"/>
       <c r="O164" s="28"/>
       <c r="P164" s="28"/>
@@ -20366,7 +20366,7 @@
       <c r="AP164" s="1"/>
       <c r="AQ164" s="14"/>
     </row>
-    <row r="165" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="165" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G165" s="1"/>
       <c r="O165" s="28"/>
       <c r="P165" s="28"/>
@@ -20377,7 +20377,7 @@
       <c r="AP165" s="1"/>
       <c r="AQ165" s="14"/>
     </row>
-    <row r="166" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="166" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G166" s="1"/>
       <c r="O166" s="28"/>
       <c r="P166" s="28"/>
@@ -20388,7 +20388,7 @@
       <c r="AP166" s="1"/>
       <c r="AQ166" s="14"/>
     </row>
-    <row r="167" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="167" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G167" s="1"/>
       <c r="O167" s="28"/>
       <c r="P167" s="28"/>
@@ -20399,7 +20399,7 @@
       <c r="AP167" s="1"/>
       <c r="AQ167" s="14"/>
     </row>
-    <row r="168" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="168" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G168" s="1"/>
       <c r="O168" s="28"/>
       <c r="P168" s="28"/>
@@ -20410,7 +20410,7 @@
       <c r="AP168" s="1"/>
       <c r="AQ168" s="14"/>
     </row>
-    <row r="169" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="169" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G169" s="1"/>
       <c r="O169" s="28"/>
       <c r="P169" s="28"/>
@@ -20421,7 +20421,7 @@
       <c r="AP169" s="1"/>
       <c r="AQ169" s="14"/>
     </row>
-    <row r="170" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="170" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G170" s="1"/>
       <c r="O170" s="28"/>
       <c r="P170" s="28"/>
@@ -20432,7 +20432,7 @@
       <c r="AP170" s="1"/>
       <c r="AQ170" s="14"/>
     </row>
-    <row r="171" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="171" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G171" s="1"/>
       <c r="O171" s="28"/>
       <c r="P171" s="28"/>
@@ -20443,7 +20443,7 @@
       <c r="AP171" s="1"/>
       <c r="AQ171" s="14"/>
     </row>
-    <row r="172" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="172" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G172" s="1"/>
       <c r="O172" s="28"/>
       <c r="P172" s="28"/>
@@ -20454,7 +20454,7 @@
       <c r="AP172" s="1"/>
       <c r="AQ172" s="14"/>
     </row>
-    <row r="173" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="173" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G173" s="1"/>
       <c r="O173" s="28"/>
       <c r="P173" s="28"/>
@@ -20465,7 +20465,7 @@
       <c r="AP173" s="1"/>
       <c r="AQ173" s="14"/>
     </row>
-    <row r="174" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="174" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G174" s="1"/>
       <c r="O174" s="28"/>
       <c r="P174" s="28"/>
@@ -20476,7 +20476,7 @@
       <c r="AP174" s="1"/>
       <c r="AQ174" s="14"/>
     </row>
-    <row r="175" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="175" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G175" s="1"/>
       <c r="O175" s="28"/>
       <c r="P175" s="28"/>
@@ -20487,7 +20487,7 @@
       <c r="AP175" s="1"/>
       <c r="AQ175" s="14"/>
     </row>
-    <row r="176" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="176" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G176" s="1"/>
       <c r="O176" s="28"/>
       <c r="P176" s="28"/>
@@ -20498,7 +20498,7 @@
       <c r="AP176" s="1"/>
       <c r="AQ176" s="14"/>
     </row>
-    <row r="177" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="177" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G177" s="1"/>
       <c r="O177" s="28"/>
       <c r="P177" s="28"/>
@@ -20509,7 +20509,7 @@
       <c r="AP177" s="1"/>
       <c r="AQ177" s="14"/>
     </row>
-    <row r="178" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="178" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G178" s="1"/>
       <c r="O178" s="28"/>
       <c r="P178" s="28"/>
@@ -20520,7 +20520,7 @@
       <c r="AP178" s="1"/>
       <c r="AQ178" s="14"/>
     </row>
-    <row r="179" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="179" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G179" s="1"/>
       <c r="O179" s="28"/>
       <c r="P179" s="28"/>
@@ -20531,7 +20531,7 @@
       <c r="AP179" s="1"/>
       <c r="AQ179" s="14"/>
     </row>
-    <row r="180" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="180" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G180" s="1"/>
       <c r="O180" s="28"/>
       <c r="P180" s="28"/>
@@ -20542,7 +20542,7 @@
       <c r="AP180" s="1"/>
       <c r="AQ180" s="14"/>
     </row>
-    <row r="181" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="181" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G181" s="1"/>
       <c r="O181" s="28"/>
       <c r="P181" s="28"/>
@@ -20553,7 +20553,7 @@
       <c r="AP181" s="1"/>
       <c r="AQ181" s="14"/>
     </row>
-    <row r="182" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="182" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G182" s="1"/>
       <c r="O182" s="28"/>
       <c r="P182" s="28"/>
@@ -20564,7 +20564,7 @@
       <c r="AP182" s="1"/>
       <c r="AQ182" s="14"/>
     </row>
-    <row r="183" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="183" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G183" s="1"/>
       <c r="O183" s="28"/>
       <c r="P183" s="28"/>
@@ -20575,7 +20575,7 @@
       <c r="AP183" s="1"/>
       <c r="AQ183" s="14"/>
     </row>
-    <row r="184" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="184" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G184" s="1"/>
       <c r="O184" s="28"/>
       <c r="P184" s="28"/>
@@ -20586,7 +20586,7 @@
       <c r="AP184" s="1"/>
       <c r="AQ184" s="14"/>
     </row>
-    <row r="185" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="185" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G185" s="1"/>
       <c r="O185" s="28"/>
       <c r="P185" s="28"/>
@@ -20597,7 +20597,7 @@
       <c r="AP185" s="1"/>
       <c r="AQ185" s="14"/>
     </row>
-    <row r="186" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="186" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G186" s="1"/>
       <c r="O186" s="28"/>
       <c r="P186" s="28"/>
@@ -20608,7 +20608,7 @@
       <c r="AP186" s="1"/>
       <c r="AQ186" s="14"/>
     </row>
-    <row r="187" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="187" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G187" s="1"/>
       <c r="O187" s="28"/>
       <c r="P187" s="28"/>
@@ -20619,7 +20619,7 @@
       <c r="AP187" s="1"/>
       <c r="AQ187" s="14"/>
     </row>
-    <row r="188" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="188" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G188" s="1"/>
       <c r="O188" s="28"/>
       <c r="P188" s="28"/>
@@ -20630,7 +20630,7 @@
       <c r="AP188" s="1"/>
       <c r="AQ188" s="14"/>
     </row>
-    <row r="189" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="189" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G189" s="1"/>
       <c r="O189" s="28"/>
       <c r="P189" s="28"/>
@@ -20641,7 +20641,7 @@
       <c r="AP189" s="1"/>
       <c r="AQ189" s="14"/>
     </row>
-    <row r="190" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="190" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G190" s="1"/>
       <c r="O190" s="28"/>
       <c r="P190" s="28"/>
@@ -20652,7 +20652,7 @@
       <c r="AP190" s="1"/>
       <c r="AQ190" s="14"/>
     </row>
-    <row r="191" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="191" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G191" s="1"/>
       <c r="O191" s="28"/>
       <c r="P191" s="28"/>
@@ -20663,7 +20663,7 @@
       <c r="AP191" s="1"/>
       <c r="AQ191" s="14"/>
     </row>
-    <row r="192" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="192" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G192" s="1"/>
       <c r="O192" s="28"/>
       <c r="P192" s="28"/>
@@ -20674,7 +20674,7 @@
       <c r="AP192" s="1"/>
       <c r="AQ192" s="14"/>
     </row>
-    <row r="193" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="193" spans="7:43" x14ac:dyDescent="0.2">
       <c r="G193" s="1"/>
       <c r="Q193" s="1"/>
       <c r="AA193" s="29"/>
@@ -20683,385 +20683,385 @@
       <c r="AP193" s="1"/>
       <c r="AQ193" s="14"/>
     </row>
-    <row r="194" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="194" spans="7:43" x14ac:dyDescent="0.2">
       <c r="Q194" s="1"/>
       <c r="AA194" s="29"/>
       <c r="AG194" s="1"/>
       <c r="AO194" s="29"/>
     </row>
-    <row r="195" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="195" spans="7:43" x14ac:dyDescent="0.2">
       <c r="Q195" s="1"/>
       <c r="AA195" s="29"/>
       <c r="AG195" s="1"/>
       <c r="AO195" s="29"/>
     </row>
-    <row r="196" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="196" spans="7:43" x14ac:dyDescent="0.2">
       <c r="Q196" s="1"/>
       <c r="AA196" s="29"/>
       <c r="AG196" s="1"/>
       <c r="AO196" s="29"/>
     </row>
-    <row r="197" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="197" spans="7:43" x14ac:dyDescent="0.2">
       <c r="Q197" s="1"/>
       <c r="AA197" s="29"/>
       <c r="AG197" s="1"/>
       <c r="AO197" s="29"/>
     </row>
-    <row r="198" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="198" spans="7:43" x14ac:dyDescent="0.2">
       <c r="Q198" s="1"/>
       <c r="AA198" s="29"/>
       <c r="AG198" s="1"/>
       <c r="AO198" s="29"/>
     </row>
-    <row r="199" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="199" spans="7:43" x14ac:dyDescent="0.2">
       <c r="Q199" s="1"/>
       <c r="AA199" s="29"/>
       <c r="AG199" s="1"/>
       <c r="AO199" s="29"/>
     </row>
-    <row r="200" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="200" spans="7:43" x14ac:dyDescent="0.2">
       <c r="Q200" s="1"/>
       <c r="AA200" s="29"/>
       <c r="AG200" s="1"/>
       <c r="AO200" s="29"/>
     </row>
-    <row r="201" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="201" spans="7:43" x14ac:dyDescent="0.2">
       <c r="Q201" s="1"/>
       <c r="AA201" s="29"/>
       <c r="AG201" s="1"/>
       <c r="AO201" s="29"/>
     </row>
-    <row r="202" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="202" spans="7:43" x14ac:dyDescent="0.2">
       <c r="Q202" s="1"/>
       <c r="AA202" s="29"/>
       <c r="AG202" s="1"/>
       <c r="AO202" s="29"/>
     </row>
-    <row r="203" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="203" spans="7:43" x14ac:dyDescent="0.2">
       <c r="Q203" s="1"/>
       <c r="AA203" s="29"/>
       <c r="AG203" s="1"/>
       <c r="AO203" s="29"/>
     </row>
-    <row r="204" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="204" spans="7:43" x14ac:dyDescent="0.2">
       <c r="Q204" s="1"/>
       <c r="AA204" s="29"/>
       <c r="AG204" s="1"/>
       <c r="AO204" s="29"/>
     </row>
-    <row r="205" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="205" spans="7:43" x14ac:dyDescent="0.2">
       <c r="Q205" s="1"/>
       <c r="AA205" s="29"/>
       <c r="AG205" s="1"/>
       <c r="AO205" s="29"/>
     </row>
-    <row r="206" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="206" spans="7:43" x14ac:dyDescent="0.2">
       <c r="Q206" s="1"/>
       <c r="AA206" s="29"/>
       <c r="AG206" s="1"/>
       <c r="AO206" s="29"/>
     </row>
-    <row r="207" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="207" spans="7:43" x14ac:dyDescent="0.2">
       <c r="Q207" s="1"/>
       <c r="AA207" s="29"/>
       <c r="AG207" s="1"/>
       <c r="AO207" s="29"/>
     </row>
-    <row r="208" spans="7:43" x14ac:dyDescent="0.3">
+    <row r="208" spans="7:43" x14ac:dyDescent="0.2">
       <c r="Q208" s="1"/>
       <c r="AA208" s="29"/>
       <c r="AG208" s="1"/>
       <c r="AO208" s="29"/>
     </row>
-    <row r="209" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="209" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q209" s="1"/>
       <c r="AA209" s="29"/>
       <c r="AG209" s="1"/>
       <c r="AO209" s="29"/>
     </row>
-    <row r="210" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="210" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q210" s="1"/>
       <c r="AA210" s="29"/>
       <c r="AG210" s="1"/>
       <c r="AO210" s="29"/>
     </row>
-    <row r="211" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="211" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q211" s="1"/>
       <c r="AA211" s="29"/>
       <c r="AG211" s="1"/>
       <c r="AO211" s="29"/>
     </row>
-    <row r="212" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="212" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q212" s="1"/>
       <c r="AA212" s="29"/>
       <c r="AG212" s="1"/>
       <c r="AO212" s="29"/>
     </row>
-    <row r="213" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="213" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q213" s="1"/>
       <c r="AA213" s="29"/>
       <c r="AG213" s="1"/>
       <c r="AO213" s="29"/>
     </row>
-    <row r="214" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="214" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q214" s="1"/>
       <c r="AA214" s="29"/>
       <c r="AG214" s="1"/>
       <c r="AO214" s="29"/>
     </row>
-    <row r="215" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="215" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q215" s="1"/>
       <c r="AA215" s="29"/>
       <c r="AG215" s="1"/>
       <c r="AO215" s="29"/>
     </row>
-    <row r="216" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="216" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q216" s="1"/>
       <c r="AA216" s="29"/>
       <c r="AG216" s="1"/>
       <c r="AO216" s="29"/>
     </row>
-    <row r="217" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="217" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q217" s="1"/>
       <c r="AA217" s="29"/>
       <c r="AG217" s="1"/>
       <c r="AO217" s="29"/>
     </row>
-    <row r="218" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="218" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q218" s="1"/>
       <c r="AA218" s="29"/>
       <c r="AG218" s="1"/>
       <c r="AO218" s="29"/>
     </row>
-    <row r="219" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="219" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q219" s="1"/>
       <c r="AA219" s="29"/>
       <c r="AG219" s="1"/>
       <c r="AO219" s="29"/>
     </row>
-    <row r="220" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="220" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q220" s="1"/>
       <c r="AA220" s="29"/>
       <c r="AG220" s="1"/>
       <c r="AO220" s="29"/>
     </row>
-    <row r="221" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="221" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q221" s="1"/>
       <c r="AA221" s="29"/>
       <c r="AG221" s="1"/>
       <c r="AO221" s="29"/>
     </row>
-    <row r="222" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="222" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q222" s="1"/>
       <c r="AA222" s="29"/>
       <c r="AG222" s="1"/>
       <c r="AO222" s="29"/>
     </row>
-    <row r="223" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="223" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q223" s="1"/>
       <c r="AA223" s="29"/>
       <c r="AG223" s="1"/>
       <c r="AO223" s="29"/>
     </row>
-    <row r="224" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="224" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q224" s="1"/>
       <c r="AA224" s="29"/>
       <c r="AG224" s="1"/>
       <c r="AO224" s="29"/>
     </row>
-    <row r="225" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="225" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q225" s="1"/>
       <c r="AA225" s="29"/>
       <c r="AG225" s="1"/>
       <c r="AO225" s="29"/>
     </row>
-    <row r="226" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="226" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q226" s="1"/>
       <c r="AA226" s="29"/>
       <c r="AG226" s="1"/>
       <c r="AO226" s="29"/>
     </row>
-    <row r="227" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="227" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q227" s="1"/>
       <c r="AA227" s="29"/>
       <c r="AG227" s="1"/>
       <c r="AO227" s="29"/>
     </row>
-    <row r="228" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="228" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q228" s="1"/>
       <c r="AA228" s="29"/>
       <c r="AG228" s="1"/>
       <c r="AO228" s="29"/>
     </row>
-    <row r="229" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="229" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q229" s="1"/>
       <c r="AA229" s="29"/>
       <c r="AG229" s="1"/>
       <c r="AO229" s="29"/>
     </row>
-    <row r="230" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="230" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q230" s="1"/>
       <c r="AA230" s="29"/>
       <c r="AG230" s="1"/>
       <c r="AO230" s="29"/>
     </row>
-    <row r="231" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="231" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q231" s="1"/>
       <c r="AA231" s="29"/>
       <c r="AG231" s="1"/>
       <c r="AO231" s="29"/>
     </row>
-    <row r="232" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="232" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q232" s="1"/>
       <c r="AA232" s="29"/>
       <c r="AG232" s="1"/>
       <c r="AO232" s="29"/>
     </row>
-    <row r="233" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="233" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q233" s="1"/>
       <c r="AA233" s="29"/>
       <c r="AG233" s="1"/>
       <c r="AO233" s="29"/>
     </row>
-    <row r="234" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="234" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q234" s="1"/>
       <c r="AA234" s="29"/>
       <c r="AG234" s="1"/>
       <c r="AO234" s="29"/>
     </row>
-    <row r="235" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="235" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q235" s="1"/>
       <c r="AA235" s="29"/>
       <c r="AG235" s="1"/>
       <c r="AO235" s="29"/>
     </row>
-    <row r="236" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="236" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q236" s="1"/>
       <c r="AA236" s="29"/>
       <c r="AG236" s="1"/>
       <c r="AO236" s="29"/>
     </row>
-    <row r="237" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="237" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q237" s="1"/>
       <c r="AA237" s="29"/>
       <c r="AG237" s="1"/>
       <c r="AO237" s="29"/>
     </row>
-    <row r="238" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="238" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q238" s="1"/>
       <c r="AA238" s="29"/>
       <c r="AG238" s="1"/>
       <c r="AO238" s="29"/>
     </row>
-    <row r="239" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="239" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q239" s="1"/>
       <c r="AA239" s="29"/>
       <c r="AG239" s="1"/>
       <c r="AO239" s="29"/>
     </row>
-    <row r="240" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="240" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q240" s="1"/>
       <c r="AA240" s="29"/>
       <c r="AG240" s="1"/>
       <c r="AO240" s="29"/>
     </row>
-    <row r="241" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="241" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q241" s="1"/>
       <c r="AA241" s="29"/>
       <c r="AG241" s="1"/>
       <c r="AO241" s="29"/>
     </row>
-    <row r="242" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="242" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q242" s="1"/>
       <c r="AA242" s="29"/>
       <c r="AG242" s="1"/>
       <c r="AO242" s="29"/>
     </row>
-    <row r="243" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="243" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q243" s="1"/>
       <c r="AA243" s="29"/>
       <c r="AG243" s="1"/>
       <c r="AO243" s="29"/>
     </row>
-    <row r="244" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="244" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q244" s="1"/>
       <c r="AA244" s="29"/>
       <c r="AG244" s="1"/>
       <c r="AO244" s="29"/>
     </row>
-    <row r="245" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="245" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q245" s="1"/>
       <c r="AA245" s="29"/>
       <c r="AG245" s="1"/>
       <c r="AO245" s="29"/>
     </row>
-    <row r="246" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="246" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q246" s="1"/>
       <c r="AA246" s="29"/>
       <c r="AG246" s="1"/>
       <c r="AO246" s="29"/>
     </row>
-    <row r="247" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="247" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q247" s="1"/>
       <c r="AA247" s="29"/>
       <c r="AG247" s="1"/>
       <c r="AO247" s="29"/>
     </row>
-    <row r="248" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="248" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q248" s="1"/>
       <c r="AA248" s="29"/>
       <c r="AG248" s="1"/>
       <c r="AO248" s="29"/>
     </row>
-    <row r="249" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="249" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q249" s="1"/>
       <c r="AA249" s="29"/>
       <c r="AG249" s="1"/>
       <c r="AO249" s="29"/>
     </row>
-    <row r="250" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="250" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q250" s="1"/>
       <c r="AA250" s="29"/>
       <c r="AG250" s="1"/>
       <c r="AO250" s="29"/>
     </row>
-    <row r="251" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="251" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q251" s="1"/>
       <c r="AA251" s="29"/>
       <c r="AG251" s="1"/>
       <c r="AO251" s="29"/>
     </row>
-    <row r="252" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="252" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q252" s="1"/>
       <c r="AA252" s="29"/>
       <c r="AG252" s="1"/>
       <c r="AO252" s="29"/>
     </row>
-    <row r="253" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="253" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q253" s="1"/>
       <c r="AA253" s="29"/>
       <c r="AG253" s="1"/>
       <c r="AO253" s="29"/>
     </row>
-    <row r="254" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="254" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q254" s="1"/>
       <c r="AA254" s="29"/>
       <c r="AG254" s="1"/>
       <c r="AO254" s="29"/>
     </row>
-    <row r="255" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="255" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q255" s="1"/>
       <c r="AA255" s="29"/>
       <c r="AG255" s="1"/>
       <c r="AO255" s="29"/>
     </row>
-    <row r="256" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="256" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q256" s="1"/>
       <c r="AA256" s="29"/>
       <c r="AG256" s="1"/>
       <c r="AO256" s="29"/>
     </row>
-    <row r="257" spans="17:41" x14ac:dyDescent="0.3">
+    <row r="257" spans="17:41" x14ac:dyDescent="0.2">
       <c r="Q257" s="1"/>
       <c r="AA257" s="29"/>
       <c r="AG257" s="1"/>

</xml_diff>